<commit_message>
feat: implement field application features, update database schema, and configure JDK environment
</commit_message>
<xml_diff>
--- a/villages_province_grade_warehouse.xlsx
+++ b/villages_province_grade_warehouse.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\laych\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\laych\Documents\digitalization_payment_dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC6A1B30-43F1-4895-8217-0A810A828D69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11B655B1-5895-4367-B807-9ED38F6F6059}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="970" yWindow="2500" windowWidth="21600" windowHeight="11180" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Village and Province" sheetId="2" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="94">
   <si>
     <t>Prey Veng</t>
   </si>
@@ -277,13 +277,40 @@
   </si>
   <si>
     <t>Other</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Whole Grain</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Broken Rice</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Impurity</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Moisture</t>
+  </si>
+  <si>
+    <t>13 - 14</t>
+  </si>
+  <si>
+    <t>13 - 15</t>
+  </si>
+  <si>
+    <t>NA</t>
+  </si>
+  <si>
+    <t>11 - 13</t>
+  </si>
+  <si>
+    <t>Foreign Matter</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -297,13 +324,24 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -318,17 +356,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyBorder="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -640,14 +681,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>61</v>
       </c>
       <c r="B1" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -671,7 +712,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -711,7 +752,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>8</v>
       </c>
@@ -719,7 +760,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>9</v>
       </c>
@@ -727,7 +768,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>10</v>
       </c>
@@ -735,7 +776,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>11</v>
       </c>
@@ -767,7 +808,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>15</v>
       </c>
@@ -775,7 +816,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>16</v>
       </c>
@@ -799,7 +840,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>19</v>
       </c>
@@ -807,7 +848,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>20</v>
       </c>
@@ -815,7 +856,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="23" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>21</v>
       </c>
@@ -823,7 +864,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>22</v>
       </c>
@@ -831,7 +872,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>23</v>
       </c>
@@ -839,7 +880,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="26" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>24</v>
       </c>
@@ -847,7 +888,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="27" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>25</v>
       </c>
@@ -855,7 +896,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="28" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>26</v>
       </c>
@@ -879,7 +920,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="31" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>29</v>
       </c>
@@ -887,7 +928,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="32" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>30</v>
       </c>
@@ -895,7 +936,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="33" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>31</v>
       </c>
@@ -903,7 +944,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="34" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
         <v>32</v>
       </c>
@@ -911,7 +952,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="35" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
         <v>33</v>
       </c>
@@ -919,7 +960,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="36" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
         <v>34</v>
       </c>
@@ -943,7 +984,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="39" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A39" s="1" t="s">
         <v>37</v>
       </c>
@@ -983,7 +1024,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="44" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A44" s="1" t="s">
         <v>42</v>
       </c>
@@ -999,7 +1040,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="46" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A46" s="1" t="s">
         <v>44</v>
       </c>
@@ -1015,7 +1056,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="48" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A48" s="1" t="s">
         <v>46</v>
       </c>
@@ -1023,7 +1064,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="49" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
         <v>47</v>
       </c>
@@ -1031,7 +1072,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="50" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A50" s="1" t="s">
         <v>48</v>
       </c>
@@ -1071,7 +1112,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="55" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A55" s="1" t="s">
         <v>53</v>
       </c>
@@ -1111,7 +1152,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="60" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A60" s="1" t="s">
         <v>58</v>
       </c>
@@ -1142,173 +1183,407 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{280BA8A1-D8D3-4E79-AA4D-67B37078E88F}">
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="29" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15" customWidth="1"/>
-    <col min="3" max="3" width="12.453125" customWidth="1"/>
+    <col min="1" max="1" width="31.36328125" customWidth="1"/>
+    <col min="2" max="2" width="10.26953125" customWidth="1"/>
+    <col min="3" max="3" width="17.453125" customWidth="1"/>
+    <col min="4" max="4" width="15.26953125" customWidth="1"/>
+    <col min="5" max="5" width="12.6328125" customWidth="1"/>
+    <col min="6" max="6" width="10.08984375" customWidth="1"/>
+    <col min="7" max="7" width="14.81640625" customWidth="1"/>
+    <col min="8" max="8" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A1" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="5" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2" s="3" t="s">
+      <c r="D1" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A2" s="2" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3" s="4"/>
+      <c r="B2" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="C2">
+        <v>1650</v>
+      </c>
+      <c r="D2">
+        <v>75</v>
+      </c>
+      <c r="E2">
+        <v>25</v>
+      </c>
+      <c r="F2">
+        <v>2</v>
+      </c>
+      <c r="G2">
+        <v>6</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
+        <v>67</v>
+      </c>
       <c r="B3" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="C3">
+        <v>1550</v>
+      </c>
+      <c r="D3">
+        <v>70</v>
+      </c>
+      <c r="E3">
+        <v>30</v>
+      </c>
+      <c r="F3">
+        <v>4</v>
+      </c>
+      <c r="G3">
+        <v>6</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="C4">
+        <v>1500</v>
+      </c>
+      <c r="D4">
+        <v>60</v>
+      </c>
+      <c r="E4">
+        <v>40</v>
+      </c>
+      <c r="F4">
+        <v>2</v>
+      </c>
+      <c r="G4">
+        <v>6</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C5">
+        <v>1450</v>
+      </c>
+      <c r="D5">
+        <v>50</v>
+      </c>
+      <c r="E5">
+        <v>50</v>
+      </c>
+      <c r="F5">
+        <v>4</v>
+      </c>
+      <c r="G5">
+        <v>6</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B6" s="4"/>
+      <c r="H6" s="3"/>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A7" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="C3">
+      <c r="C7">
+        <v>1850</v>
+      </c>
+      <c r="D7">
+        <v>75</v>
+      </c>
+      <c r="E7">
+        <v>25</v>
+      </c>
+      <c r="F7" t="s">
+        <v>91</v>
+      </c>
+      <c r="G7">
+        <v>6</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A8" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="C8">
+        <v>1750</v>
+      </c>
+      <c r="D8">
+        <v>70</v>
+      </c>
+      <c r="E8">
+        <v>30</v>
+      </c>
+      <c r="F8" t="s">
+        <v>91</v>
+      </c>
+      <c r="G8">
+        <v>6</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A9" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="C9">
+        <v>1700</v>
+      </c>
+      <c r="D9">
+        <v>60</v>
+      </c>
+      <c r="E9">
+        <v>40</v>
+      </c>
+      <c r="F9" t="s">
+        <v>91</v>
+      </c>
+      <c r="G9">
+        <v>6</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A10" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C10">
         <v>1650</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A4" s="4"/>
-      <c r="B4" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="C4">
-        <v>1550</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A5" s="4"/>
-      <c r="B5" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="C5">
-        <v>1500</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A6" s="4"/>
-      <c r="B6" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="C6">
-        <v>1450</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A8" s="3" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A9" s="4"/>
-      <c r="B9" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="C9">
-        <v>1850</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A10" s="4"/>
-      <c r="B10" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="C10">
-        <v>1750</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A11" s="4"/>
-      <c r="B11" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="C11">
-        <v>1700</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A12" s="4"/>
+      <c r="D10">
+        <v>50</v>
+      </c>
+      <c r="E10">
+        <v>50</v>
+      </c>
+      <c r="F10" t="s">
+        <v>91</v>
+      </c>
+      <c r="G10">
+        <v>6</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A11" s="2"/>
+      <c r="B11" s="4"/>
+      <c r="H11" s="3"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A12" s="2" t="s">
+        <v>70</v>
+      </c>
       <c r="B12" s="4" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C12">
-        <v>1650</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A13" s="3" t="s">
+        <v>2150</v>
+      </c>
+      <c r="D12">
+        <v>98</v>
+      </c>
+      <c r="E12" t="s">
+        <v>91</v>
+      </c>
+      <c r="F12">
+        <v>1</v>
+      </c>
+      <c r="G12">
+        <v>1</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A13" s="2"/>
+      <c r="B13" s="4"/>
+      <c r="H13" s="3"/>
+    </row>
+    <row r="14" spans="1:8" ht="14" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="2" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A14" s="4"/>
       <c r="B14" s="4" t="s">
         <v>78</v>
       </c>
       <c r="C14">
         <v>2050</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A16" s="3" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A17" s="4"/>
-      <c r="B17" t="s">
+      <c r="D14">
+        <v>98</v>
+      </c>
+      <c r="E14" t="s">
+        <v>91</v>
+      </c>
+      <c r="F14">
+        <v>1</v>
+      </c>
+      <c r="G14">
+        <v>1</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B15" s="4"/>
+      <c r="H15" s="3"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A16" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B16" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="C17">
-        <v>2150</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A19" s="3" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A20" s="4"/>
-      <c r="B20" t="s">
+      <c r="C16">
+        <v>1900</v>
+      </c>
+      <c r="D16">
+        <v>96</v>
+      </c>
+      <c r="E16" t="s">
+        <v>91</v>
+      </c>
+      <c r="F16">
+        <v>2</v>
+      </c>
+      <c r="G16">
+        <v>2</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B17" s="4"/>
+      <c r="H17" s="3"/>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A18" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B18" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="C20">
-        <v>1900</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A22" s="3" t="s">
+      <c r="C18">
+        <v>1320</v>
+      </c>
+      <c r="D18" t="s">
+        <v>91</v>
+      </c>
+      <c r="E18" t="s">
+        <v>91</v>
+      </c>
+      <c r="F18" t="s">
+        <v>91</v>
+      </c>
+      <c r="G18">
+        <v>4</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A19" s="2" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A23" s="4"/>
-      <c r="B23" t="s">
-        <v>78</v>
-      </c>
-      <c r="C23">
-        <v>1320</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A24" s="4"/>
-      <c r="B24" t="s">
+      <c r="B19" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="C24">
+      <c r="C19">
         <v>1220</v>
       </c>
+      <c r="D19" t="s">
+        <v>91</v>
+      </c>
+      <c r="E19" t="s">
+        <v>91</v>
+      </c>
+      <c r="F19" t="s">
+        <v>91</v>
+      </c>
+      <c r="G19">
+        <v>8</v>
+      </c>
+      <c r="H19" s="3" t="s">
+        <v>89</v>
+      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>